<commit_message>
Aktualizacja narzedzi Beast Feast (2026-09-26 01:10)
</commit_message>
<xml_diff>
--- a/Beast_Feast_Adversaries_Environments.xlsx
+++ b/Beast_Feast_Adversaries_Environments.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adversaries" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Umiejętności" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Legenda" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Adversaries" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Environments" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Umiejętności" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Adversaries'!$A$1:$L$268</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Adversaries'!$A$1:$L$291</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environments'!$A$1:$H$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Umiejętności'!$A$1:$Z$826</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Umiejętności'!$A$1:$Z$869</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -769,7 +769,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
@@ -858,6 +857,63 @@
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">    warto zweryfikować z oryginalnym eksportem z Daggerheart encounter manager (FreshCutGrass.app).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>KOLOSY (Core Rulebook — Colossus of the Drylands, s. 318–327)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 23 karty w arkuszu "Adversaries" z podtypem "Colossus": 4 kolosy (Ikeri T1, Daktadae T2, Poy T3, Kelir T4),</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    każdy jako karta "&lt;Nazwa&gt;: Framework" + osobne karty segmentów ("Ikeri: Head", "Ikeri: Arm ×2" itd.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Framework = wspólne progi, Stress i cechy całego kolosa; Difficulty frameworku = najwyższa z segmentów.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Segmenty mają skopiowane progi frameworku; "×2" w nazwie = tyle sztuk segmentu (każda z osobnym HP).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Nazwy bez przecinków celowo — kolumna "Źródła" w "Umiejętności" rozdziela nazwy przecinkami.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 43 nowych rodzin umiejętności w kategorii "Kolosy" (w tym 12 przykładowych cech kolosów z podręcznika),</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    a istniejące rodziny Crush, Flying dostały nowe warianty.</t>
         </is>
       </c>
     </row>
@@ -872,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L268"/>
+  <dimension ref="A1:L291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16715,8 +16771,1166 @@
         </is>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B269" s="12" t="inlineStr">
+        <is>
+          <t>Ikeri: Framework</t>
+        </is>
+      </c>
+      <c r="C269" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D269" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E269" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri, Injuries Untold — framework kolosa. This apelike creature has the face of a bird. They are made of stone and carry an enormous mesa upon their back. Size: 95 ft. tall, 60 ft. wide. Segments: 2 Legs, 2 Arms, 1 Torso, and 1 Head. Framework trzyma wspólne progi, Stress i cechy całego kolosa; Difficulty = najwyższa z segmentów (dla efektów celujących w całego kolosa).</t>
+        </is>
+      </c>
+      <c r="F269" s="8" t="inlineStr">
+        <is>
+          <t>Entangle, intimidate, peck, stomp</t>
+        </is>
+      </c>
+      <c r="G269" s="12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H269" s="12" t="inlineStr">
+        <is>
+          <t>11/22</t>
+        </is>
+      </c>
+      <c r="I269" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J269" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K269" s="8" t="n"/>
+      <c r="L269" s="8" t="inlineStr">
+        <is>
+          <t>Eagle Eyes +3, Huge +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B270" s="12" t="inlineStr">
+        <is>
+          <t>Ikeri: Head</t>
+        </is>
+      </c>
+      <c r="C270" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D270" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E270" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Ikeri, Injuries Untold. Adjacent Segments: Torso. Progi i Stress wspólne — z karty „Ikeri: Framework”.</t>
+        </is>
+      </c>
+      <c r="F270" s="8" t="n"/>
+      <c r="G270" s="12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H270" s="12" t="inlineStr">
+        <is>
+          <t>11/22</t>
+        </is>
+      </c>
+      <c r="I270" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J270" s="12" t="n"/>
+      <c r="K270" s="8" t="inlineStr">
+        <is>
+          <t>+2 | Peck: Melee | 1d10+1 phy</t>
+        </is>
+      </c>
+      <c r="L270" s="8" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B271" s="12" t="inlineStr">
+        <is>
+          <t>Ikeri: Torso</t>
+        </is>
+      </c>
+      <c r="C271" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D271" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E271" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Ikeri, Injuries Untold. Adjacent Segments: Head, Arms, Legs. Progi i Stress wspólne — z karty „Ikeri: Framework”.</t>
+        </is>
+      </c>
+      <c r="F271" s="8" t="n"/>
+      <c r="G271" s="12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H271" s="12" t="inlineStr">
+        <is>
+          <t>11/22</t>
+        </is>
+      </c>
+      <c r="I271" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J271" s="12" t="n"/>
+      <c r="K271" s="8" t="n"/>
+      <c r="L271" s="8" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B272" s="12" t="inlineStr">
+        <is>
+          <t>Ikeri: Arm ×2</t>
+        </is>
+      </c>
+      <c r="C272" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D272" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E272" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Ikeri, Injuries Untold. Występuje 2× — dodaj 2 instancje, HP liczone osobno dla każdej. Adjacent Segments: Torso. Progi i Stress wspólne — z karty „Ikeri: Framework”.</t>
+        </is>
+      </c>
+      <c r="F272" s="8" t="n"/>
+      <c r="G272" s="12" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H272" s="12" t="inlineStr">
+        <is>
+          <t>11/22</t>
+        </is>
+      </c>
+      <c r="I272" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J272" s="12" t="n"/>
+      <c r="K272" s="8" t="inlineStr">
+        <is>
+          <t>+2 | Punch: Very Close | 1d8+6 phy</t>
+        </is>
+      </c>
+      <c r="L272" s="8" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B273" s="12" t="inlineStr">
+        <is>
+          <t>Ikeri: Leg ×2</t>
+        </is>
+      </c>
+      <c r="C273" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D273" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E273" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Ikeri, Injuries Untold. Występuje 2× — dodaj 2 instancje, HP liczone osobno dla każdej. Adjacent Segments: Torso, Leg. Progi i Stress wspólne — z karty „Ikeri: Framework”.</t>
+        </is>
+      </c>
+      <c r="F273" s="8" t="n"/>
+      <c r="G273" s="12" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H273" s="12" t="inlineStr">
+        <is>
+          <t>11/22</t>
+        </is>
+      </c>
+      <c r="I273" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J273" s="12" t="n"/>
+      <c r="K273" s="8" t="inlineStr">
+        <is>
+          <t>+2 | Stomp: Very Close | 1d6+3 phy</t>
+        </is>
+      </c>
+      <c r="L273" s="8" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B274" s="12" t="inlineStr">
+        <is>
+          <t>Daktadae: Framework</t>
+        </is>
+      </c>
+      <c r="C274" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D274" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E274" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae, the Cleaver — framework kolosa. A massive steel rhinoceros formed from a steam train, a cleaver emerging from his head instead of a horn. Size: 130 ft. tall, 220 ft. long. Segments: 2 Forelegs, 2 Hindlegs, 1 Torso, and 1 Head. Framework trzyma wspólne progi, Stress i cechy całego kolosa; Difficulty = najwyższa z segmentów (dla efektów celujących w całego kolosa).</t>
+        </is>
+      </c>
+      <c r="F274" s="8" t="inlineStr">
+        <is>
+          <t>Clear forests, cleave, hew, stomp</t>
+        </is>
+      </c>
+      <c r="G274" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H274" s="12" t="inlineStr">
+        <is>
+          <t>16/25</t>
+        </is>
+      </c>
+      <c r="I274" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J274" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K274" s="8" t="n"/>
+      <c r="L274" s="8" t="inlineStr">
+        <is>
+          <t>Huge +2, Trampling +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B275" s="12" t="inlineStr">
+        <is>
+          <t>Daktadae: Head</t>
+        </is>
+      </c>
+      <c r="C275" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D275" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E275" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Daktadae, the Cleaver. Adjacent Segments: Torso. Progi i Stress wspólne — z karty „Daktadae: Framework”.</t>
+        </is>
+      </c>
+      <c r="F275" s="8" t="n"/>
+      <c r="G275" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H275" s="12" t="inlineStr">
+        <is>
+          <t>16/25</t>
+        </is>
+      </c>
+      <c r="I275" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J275" s="12" t="n"/>
+      <c r="K275" s="8" t="inlineStr">
+        <is>
+          <t>+2 | Cleaver: Melee | 2d20+8 phy</t>
+        </is>
+      </c>
+      <c r="L275" s="8" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B276" s="12" t="inlineStr">
+        <is>
+          <t>Daktadae: Torso</t>
+        </is>
+      </c>
+      <c r="C276" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D276" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E276" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Daktadae, the Cleaver. Adjacent Segments: Head, Forelegs, Hindlegs. Progi i Stress wspólne — z karty „Daktadae: Framework”.</t>
+        </is>
+      </c>
+      <c r="F276" s="8" t="n"/>
+      <c r="G276" s="12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H276" s="12" t="inlineStr">
+        <is>
+          <t>16/25</t>
+        </is>
+      </c>
+      <c r="I276" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J276" s="12" t="n"/>
+      <c r="K276" s="8" t="n"/>
+      <c r="L276" s="8" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B277" s="12" t="inlineStr">
+        <is>
+          <t>Daktadae: Foreleg ×2</t>
+        </is>
+      </c>
+      <c r="C277" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D277" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E277" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Daktadae, the Cleaver. Występuje 2× — dodaj 2 instancje, HP liczone osobno dla każdej. Adjacent Segments: Torso, Forelegs. Progi i Stress wspólne — z karty „Daktadae: Framework”.</t>
+        </is>
+      </c>
+      <c r="F277" s="8" t="n"/>
+      <c r="G277" s="12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H277" s="12" t="inlineStr">
+        <is>
+          <t>16/25</t>
+        </is>
+      </c>
+      <c r="I277" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J277" s="12" t="n"/>
+      <c r="K277" s="8" t="inlineStr">
+        <is>
+          <t>+1 | Stomp: Very Close | 2d10+8 phy</t>
+        </is>
+      </c>
+      <c r="L277" s="8" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B278" s="12" t="inlineStr">
+        <is>
+          <t>Daktadae: Hindleg ×2</t>
+        </is>
+      </c>
+      <c r="C278" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D278" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E278" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Daktadae, the Cleaver. Występuje 2× — dodaj 2 instancje, HP liczone osobno dla każdej. Adjacent Segments: Torso, Hindlegs. Progi i Stress wspólne — z karty „Daktadae: Framework”.</t>
+        </is>
+      </c>
+      <c r="F278" s="8" t="n"/>
+      <c r="G278" s="12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H278" s="12" t="inlineStr">
+        <is>
+          <t>16/25</t>
+        </is>
+      </c>
+      <c r="I278" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J278" s="12" t="n"/>
+      <c r="K278" s="8" t="inlineStr">
+        <is>
+          <t>+1 | Stomp: Very Close | 2d10+8 phy</t>
+        </is>
+      </c>
+      <c r="L278" s="8" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B279" s="12" t="inlineStr">
+        <is>
+          <t>Poy: Framework</t>
+        </is>
+      </c>
+      <c r="C279" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D279" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E279" s="8" t="inlineStr">
+        <is>
+          <t>Poy, Sky Skimmer of the Dust Sea — framework kolosa. This massive shoebill stork is formed from the dust of the Drylands and traps enemies in their cavernous beak. Size: 220 ft. long, 160 ft. wingspan. Segments: 1 Head, 1 Neck, 2 Wings, 1 Body, 2 Talons, 1 Tail. Framework trzyma wspólne progi, Stress i cechy całego kolosa; Difficulty = najwyższa z segmentów (dla efektów celujących w całego kolosa).</t>
+        </is>
+      </c>
+      <c r="F279" s="8" t="inlineStr">
+        <is>
+          <t>Corral, intimidate, maintain distance</t>
+        </is>
+      </c>
+      <c r="G279" s="12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H279" s="12" t="inlineStr">
+        <is>
+          <t>25/48</t>
+        </is>
+      </c>
+      <c r="I279" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J279" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K279" s="8" t="n"/>
+      <c r="L279" s="8" t="inlineStr">
+        <is>
+          <t>Attack From Above +3, Huge +3, Maneuver +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B280" s="12" t="inlineStr">
+        <is>
+          <t>Poy: Head</t>
+        </is>
+      </c>
+      <c r="C280" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D280" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E280" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Poy, Sky Skimmer of the Dust Sea. Adjacent Segments: Neck. Progi i Stress wspólne — z karty „Poy: Framework”.</t>
+        </is>
+      </c>
+      <c r="F280" s="8" t="n"/>
+      <c r="G280" s="12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H280" s="12" t="inlineStr">
+        <is>
+          <t>25/48</t>
+        </is>
+      </c>
+      <c r="I280" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J280" s="12" t="n"/>
+      <c r="K280" s="8" t="inlineStr">
+        <is>
+          <t>+3 | Screech: Very Far | 3d8+2 mag</t>
+        </is>
+      </c>
+      <c r="L280" s="8" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B281" s="12" t="inlineStr">
+        <is>
+          <t>Poy: Neck</t>
+        </is>
+      </c>
+      <c r="C281" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D281" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E281" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Poy, Sky Skimmer of the Dust Sea. Adjacent Segments: Head, Body. Progi i Stress wspólne — z karty „Poy: Framework”.</t>
+        </is>
+      </c>
+      <c r="F281" s="8" t="n"/>
+      <c r="G281" s="12" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H281" s="12" t="inlineStr">
+        <is>
+          <t>25/48</t>
+        </is>
+      </c>
+      <c r="I281" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J281" s="12" t="n"/>
+      <c r="K281" s="8" t="n"/>
+      <c r="L281" s="8" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B282" s="12" t="inlineStr">
+        <is>
+          <t>Poy: Wing ×2</t>
+        </is>
+      </c>
+      <c r="C282" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D282" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E282" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Poy, Sky Skimmer of the Dust Sea. Występuje 2× — dodaj 2 instancje, HP liczone osobno dla każdej. Adjacent Segments: Body. Progi i Stress wspólne — z karty „Poy: Framework”.</t>
+        </is>
+      </c>
+      <c r="F282" s="8" t="n"/>
+      <c r="G282" s="12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H282" s="12" t="inlineStr">
+        <is>
+          <t>25/48</t>
+        </is>
+      </c>
+      <c r="I282" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J282" s="12" t="n"/>
+      <c r="K282" s="8" t="inlineStr">
+        <is>
+          <t>+2 | Swipe: Melee | 3d12+9 phy</t>
+        </is>
+      </c>
+      <c r="L282" s="8" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B283" s="12" t="inlineStr">
+        <is>
+          <t>Poy: Body</t>
+        </is>
+      </c>
+      <c r="C283" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D283" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E283" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Poy, Sky Skimmer of the Dust Sea. Adjacent Segments: Wings, Neck, Tail, Talons. Progi i Stress wspólne — z karty „Poy: Framework”.</t>
+        </is>
+      </c>
+      <c r="F283" s="8" t="n"/>
+      <c r="G283" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H283" s="12" t="inlineStr">
+        <is>
+          <t>25/48</t>
+        </is>
+      </c>
+      <c r="I283" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J283" s="12" t="n"/>
+      <c r="K283" s="8" t="n"/>
+      <c r="L283" s="8" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B284" s="12" t="inlineStr">
+        <is>
+          <t>Poy: Talon ×2</t>
+        </is>
+      </c>
+      <c r="C284" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D284" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E284" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Poy, Sky Skimmer of the Dust Sea. Występuje 2× — dodaj 2 instancje, HP liczone osobno dla każdej. Adjacent Segments: Body, Tail. Progi i Stress wspólne — z karty „Poy: Framework”.</t>
+        </is>
+      </c>
+      <c r="F284" s="8" t="n"/>
+      <c r="G284" s="12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H284" s="12" t="inlineStr">
+        <is>
+          <t>25/48</t>
+        </is>
+      </c>
+      <c r="I284" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J284" s="12" t="n"/>
+      <c r="K284" s="8" t="inlineStr">
+        <is>
+          <t>+2 | Talon Strike: Melee | 3d10+5 phy</t>
+        </is>
+      </c>
+      <c r="L284" s="8" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B285" s="12" t="inlineStr">
+        <is>
+          <t>Poy: Tail</t>
+        </is>
+      </c>
+      <c r="C285" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D285" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E285" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Poy, Sky Skimmer of the Dust Sea. Adjacent Segments: Body, Talons. Progi i Stress wspólne — z karty „Poy: Framework”.</t>
+        </is>
+      </c>
+      <c r="F285" s="8" t="n"/>
+      <c r="G285" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H285" s="12" t="inlineStr">
+        <is>
+          <t>25/48</t>
+        </is>
+      </c>
+      <c r="I285" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J285" s="12" t="n"/>
+      <c r="K285" s="8" t="inlineStr">
+        <is>
+          <t>+1 | Whip: Very Close | 3d12+12 phy</t>
+        </is>
+      </c>
+      <c r="L285" s="8" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B286" s="12" t="inlineStr">
+        <is>
+          <t>Kelir: Framework</t>
+        </is>
+      </c>
+      <c r="C286" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D286" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E286" s="8" t="inlineStr">
+        <is>
+          <t>Kelir, the Virulent Hate &amp; Her Hundred, Hundred Children — framework kolosa. A crablike, mountainous beast whose children scurry in and around her, bringing food as tribute. Size: 275 ft. tall, 150 ft. wide. Segments: 1 Head, 1 Shell, 1 Body Cavity, 2 Claws, and 4 Legs. Framework trzyma wspólne progi, Stress i cechy całego kolosa; Difficulty = najwyższa z segmentów (dla efektów celujących w całego kolosa).</t>
+        </is>
+      </c>
+      <c r="F286" s="8" t="inlineStr">
+        <is>
+          <t>Consume, ravage, swarm</t>
+        </is>
+      </c>
+      <c r="G286" s="12" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="H286" s="12" t="inlineStr">
+        <is>
+          <t>30/65</t>
+        </is>
+      </c>
+      <c r="I286" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J286" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K286" s="8" t="n"/>
+      <c r="L286" s="8" t="inlineStr">
+        <is>
+          <t>Contempt +2, Huge +4, Sense Movement +4</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B287" s="12" t="inlineStr">
+        <is>
+          <t>Kelir: Head</t>
+        </is>
+      </c>
+      <c r="C287" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D287" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E287" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Kelir, the Virulent Hate &amp; Her Hundred, Hundred Children. Adjacent Segments: Body. Progi i Stress wspólne — z karty „Kelir: Framework”.</t>
+        </is>
+      </c>
+      <c r="F287" s="8" t="n"/>
+      <c r="G287" s="12" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="H287" s="12" t="inlineStr">
+        <is>
+          <t>30/65</t>
+        </is>
+      </c>
+      <c r="I287" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J287" s="12" t="n"/>
+      <c r="K287" s="8" t="inlineStr">
+        <is>
+          <t>+4 | Eye Beams: Close | 4d6+6 mag</t>
+        </is>
+      </c>
+      <c r="L287" s="8" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B288" s="12" t="inlineStr">
+        <is>
+          <t>Kelir: Shell</t>
+        </is>
+      </c>
+      <c r="C288" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D288" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E288" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Kelir, the Virulent Hate &amp; Her Hundred, Hundred Children. Adjacent Segments: Head, Legs, Claws, Body Cavity. Progi i Stress wspólne — z karty „Kelir: Framework”.</t>
+        </is>
+      </c>
+      <c r="F288" s="8" t="n"/>
+      <c r="G288" s="12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H288" s="12" t="inlineStr">
+        <is>
+          <t>30/65</t>
+        </is>
+      </c>
+      <c r="I288" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J288" s="12" t="n"/>
+      <c r="K288" s="8" t="n"/>
+      <c r="L288" s="8" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B289" s="12" t="inlineStr">
+        <is>
+          <t>Kelir: Body Cavity</t>
+        </is>
+      </c>
+      <c r="C289" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D289" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E289" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Kelir, the Virulent Hate &amp; Her Hundred, Hundred Children. Adjacent Segments: Shell. Progi i Stress wspólne — z karty „Kelir: Framework”.</t>
+        </is>
+      </c>
+      <c r="F289" s="8" t="n"/>
+      <c r="G289" s="12" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="H289" s="12" t="inlineStr">
+        <is>
+          <t>30/65</t>
+        </is>
+      </c>
+      <c r="I289" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J289" s="12" t="n"/>
+      <c r="K289" s="8" t="n"/>
+      <c r="L289" s="8" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B290" s="12" t="inlineStr">
+        <is>
+          <t>Kelir: Claw ×2</t>
+        </is>
+      </c>
+      <c r="C290" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D290" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E290" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Kelir, the Virulent Hate &amp; Her Hundred, Hundred Children. Występuje 2× — dodaj 2 instancje, HP liczone osobno dla każdej. Adjacent Segments: Shell. Progi i Stress wspólne — z karty „Kelir: Framework”.</t>
+        </is>
+      </c>
+      <c r="F290" s="8" t="n"/>
+      <c r="G290" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H290" s="12" t="inlineStr">
+        <is>
+          <t>30/65</t>
+        </is>
+      </c>
+      <c r="I290" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J290" s="12" t="n"/>
+      <c r="K290" s="8" t="inlineStr">
+        <is>
+          <t>+5 | Pincer: Very Close | 3d20+8 phy</t>
+        </is>
+      </c>
+      <c r="L290" s="8" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B291" s="12" t="inlineStr">
+        <is>
+          <t>Kelir: Leg ×4</t>
+        </is>
+      </c>
+      <c r="C291" s="12" t="inlineStr">
+        <is>
+          <t>Colossus</t>
+        </is>
+      </c>
+      <c r="D291" s="12" t="inlineStr">
+        <is>
+          <t>Core Rulebook (Colossus of the Drylands)</t>
+        </is>
+      </c>
+      <c r="E291" s="8" t="inlineStr">
+        <is>
+          <t>Segment kolosa Kelir, the Virulent Hate &amp; Her Hundred, Hundred Children. Występuje 4× — dodaj 4 instancje, HP liczone osobno dla każdej. Adjacent Segments: Shell. Progi i Stress wspólne — z karty „Kelir: Framework”.</t>
+        </is>
+      </c>
+      <c r="F291" s="8" t="n"/>
+      <c r="G291" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H291" s="12" t="inlineStr">
+        <is>
+          <t>30/65</t>
+        </is>
+      </c>
+      <c r="I291" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J291" s="12" t="n"/>
+      <c r="K291" s="8" t="inlineStr">
+        <is>
+          <t>+4 | Stomp: Very Close | 4d10+6 phy</t>
+        </is>
+      </c>
+      <c r="L291" s="8" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L268"/>
+  <autoFilter ref="A1:L291"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18674,7 +19888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z826"/>
+  <dimension ref="A1:Z869"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21252,10 +22466,16 @@
           <t>Mark a Stress to deal 2d6+8 direct physical damage to a target with 3 or more bramble tokens.</t>
         </is>
       </c>
-      <c r="F56" s="12" t="n"/>
+      <c r="F56" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
       <c r="G56" s="12" t="n"/>
-      <c r="H56" s="12" t="n">
-        <v>2</v>
+      <c r="H56" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="I56" s="12" t="inlineStr">
         <is>
@@ -21264,12 +22484,17 @@
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t>Giant Octopus, Tangle Bramble Swarm</t>
+          <t>Giant Octopus, Tangle Bramble Swarm, Ikeri: Arm ×2</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
           <t>[Crush] Mark a Stress to deal 3d8 direct physical damage to a target Grappled by the &lt;Adversary&gt;.  (Źródła: Giant Octopus)</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>[Crush] Spend a Fear to make an attack against a target on another segment of Ikeri. On a success, Ikeri grabs and crushes the target, dealing 1d20+4 physical damage and Restraining them until this Arm takes Major or greater damage. When this Arm takes the spotlight while the target is still in Ikeri’s hand, the target takes 1d20 physical damage.  (Źródła: Ikeri: Arm ×2)</t>
         </is>
       </c>
     </row>
@@ -40872,8 +42097,10 @@
       </c>
       <c r="F494" s="12" t="n"/>
       <c r="G494" s="12" t="n"/>
-      <c r="H494" s="12" t="n">
-        <v>9</v>
+      <c r="H494" s="12" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="I494" s="12" t="inlineStr">
         <is>
@@ -40882,7 +42109,7 @@
       </c>
       <c r="J494" s="8" t="inlineStr">
         <is>
-          <t>Ashen Tyrant, Dire Bat, Falcon, Giant Eagle, Giant Mosquitoes, Manticore, Obsidian Predator, Rugaru, Vampire Lord</t>
+          <t>Ashen Tyrant, Dire Bat, Falcon, Giant Eagle, Giant Mosquitoes, Manticore, Obsidian Predator, Rugaru, Vampire Lord, Poy: Framework</t>
         </is>
       </c>
       <c r="K494" t="inlineStr">
@@ -40913,6 +42140,11 @@
       <c r="P494" t="inlineStr">
         <is>
           <t>[On Crimson Wings] While flying, the Hellwing gains a +1 bonus to their Difficulty.  (Źródła: Vampire Lord)</t>
+        </is>
+      </c>
+      <c r="Q494" t="inlineStr">
+        <is>
+          <t>[Flying] Poy can fly unless one of their Wings is Destroyed. While Poy is flying, each segment’s Difficulty gains a +2 bonus against action rolls made by PCs who aren’t on Poy.  (Źródła: Poy: Framework)</t>
         </is>
       </c>
     </row>
@@ -55495,8 +56727,2067 @@
         </is>
       </c>
     </row>
+    <row r="827">
+      <c r="A827" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B827" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C827" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D827" s="8" t="inlineStr">
+        <is>
+          <t>Fatal</t>
+        </is>
+      </c>
+      <c r="E827" s="8" t="inlineStr">
+        <is>
+          <t>When this segment is Destroyed, the colossus is defeated.</t>
+        </is>
+      </c>
+      <c r="F827" s="12" t="n"/>
+      <c r="G827" s="12" t="n"/>
+      <c r="H827" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I827" s="12" t="inlineStr">
+        <is>
+          <t>1,2,3,4</t>
+        </is>
+      </c>
+      <c r="J827" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Head, Ikeri: Torso, Daktadae: Torso, Poy: Neck, Kelir: Body Cavity</t>
+        </is>
+      </c>
+      <c r="K827" t="inlineStr">
+        <is>
+          <t>[Fatal] When the Head is Destroyed, Ikeri is defeated.  (Źródła: Ikeri: Head)</t>
+        </is>
+      </c>
+      <c r="L827" t="inlineStr">
+        <is>
+          <t>[Fatal] When the Torso is Destroyed, Ikeri is defeated.  (Źródła: Ikeri: Torso)</t>
+        </is>
+      </c>
+      <c r="M827" t="inlineStr">
+        <is>
+          <t>[Fatal] When this segment is Destroyed, Daktadae is defeated.  (Źródła: Daktadae: Torso)</t>
+        </is>
+      </c>
+      <c r="N827" t="inlineStr">
+        <is>
+          <t>[Fatal] When this segment is Destroyed, Poy is defeated.  (Źródła: Poy: Neck)</t>
+        </is>
+      </c>
+      <c r="O827" t="inlineStr">
+        <is>
+          <t>[Fatal] If this segment is Destroyed, Kelir is defeated.  (Źródła: Kelir: Body Cavity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B828" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C828" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D828" s="8" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E828" s="8" t="inlineStr">
+        <is>
+          <t>When all segments in this chain are Destroyed, the colossus is defeated.</t>
+        </is>
+      </c>
+      <c r="F828" s="12" t="n"/>
+      <c r="G828" s="12" t="n"/>
+      <c r="H828" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I828" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J828" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Arm ×2, Ikeri: Leg ×2</t>
+        </is>
+      </c>
+      <c r="K828" t="inlineStr">
+        <is>
+          <t>[Chain (A)] When all segments in Chain A are Destroyed, Ikeri is defeated.  (Źródła: Ikeri: Arm ×2, Ikeri: Leg ×2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B829" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C829" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D829" s="8" t="inlineStr">
+        <is>
+          <t>Strike (Melee)</t>
+        </is>
+      </c>
+      <c r="E829" s="8" t="inlineStr">
+        <is>
+          <t>This segment is immune to damage from attacks not made within Melee range.</t>
+        </is>
+      </c>
+      <c r="F829" s="12" t="n"/>
+      <c r="G829" s="12" t="n"/>
+      <c r="H829" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I829" s="12" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="J829" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Head, Kelir: Head, Kelir: Claw ×2</t>
+        </is>
+      </c>
+      <c r="K829" t="inlineStr">
+        <is>
+          <t>[Strike (Melee)] The Head is immune to damage from attacks not made within Melee range.  (Źródła: Ikeri: Head)</t>
+        </is>
+      </c>
+      <c r="L829" t="inlineStr">
+        <is>
+          <t>[Strike (Very Close)] The Head is immune to damage from attacks not made within Very Close range.  (Źródła: Kelir: Head)</t>
+        </is>
+      </c>
+      <c r="M829" t="inlineStr">
+        <is>
+          <t>[Strike (Very Close)] The Claws are immune to damage from attacks not made within Very Close range.  (Źródła: Kelir: Claw ×2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B830" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C830" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D830" s="8" t="inlineStr">
+        <is>
+          <t>Armored</t>
+        </is>
+      </c>
+      <c r="E830" s="8" t="inlineStr">
+        <is>
+          <t>When this segment marks HP from an attack, it marks 1 fewer HP.</t>
+        </is>
+      </c>
+      <c r="F830" s="12" t="n"/>
+      <c r="G830" s="12" t="n"/>
+      <c r="H830" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I830" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J830" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Shell</t>
+        </is>
+      </c>
+      <c r="K830" t="inlineStr">
+        <is>
+          <t>[Armored] When the Shell marks HP from an attack, it marks 1 fewer HP.  (Źródła: Kelir: Shell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B831" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C831" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D831" s="8" t="inlineStr">
+        <is>
+          <t>Climbing (+3)</t>
+        </is>
+      </c>
+      <c r="E831" s="8" t="inlineStr">
+        <is>
+          <t>This segment’s Difficulty gains a +3 bonus against action rolls made to climb it.</t>
+        </is>
+      </c>
+      <c r="F831" s="12" t="n"/>
+      <c r="G831" s="12" t="n"/>
+      <c r="H831" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I831" s="12" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="J831" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Torso, Kelir: Leg ×4</t>
+        </is>
+      </c>
+      <c r="K831" t="inlineStr">
+        <is>
+          <t>[Climbing (+3)] The Torso’s Difficulty gains a +3 bonus against action rolls made to climb it unless the Head is Broken.  (Źródła: Daktadae: Torso)</t>
+        </is>
+      </c>
+      <c r="L831" t="inlineStr">
+        <is>
+          <t>[Climbing (−2)] An action roll made to climb on the leg gains a −2 penalty to its Difficulty.  (Źródła: Kelir: Leg ×4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B832" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C832" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D832" s="8" t="inlineStr">
+        <is>
+          <t>Not Climbable</t>
+        </is>
+      </c>
+      <c r="E832" s="8" t="inlineStr">
+        <is>
+          <t>This segment can’t be climbed.</t>
+        </is>
+      </c>
+      <c r="F832" s="12" t="n"/>
+      <c r="G832" s="12" t="n"/>
+      <c r="H832" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I832" s="12" t="n"/>
+      <c r="J832" s="8" t="inlineStr">
+        <is>
+          <t>Colossus of the Drylands (przykład)</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B833" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C833" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D833" s="8" t="inlineStr">
+        <is>
+          <t>Weak Point</t>
+        </is>
+      </c>
+      <c r="E833" s="8" t="inlineStr">
+        <is>
+          <t>The colossus has a weak point on this segment. When this segment marks HP from an attack made within Melee range, it marks an additional HP.</t>
+        </is>
+      </c>
+      <c r="F833" s="12" t="n"/>
+      <c r="G833" s="12" t="n"/>
+      <c r="H833" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I833" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J833" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Torso</t>
+        </is>
+      </c>
+      <c r="K833" t="inlineStr">
+        <is>
+          <t>[Weak Point] The underbelly of the Torso has a weak point. When this segment marks HP from an attack within Melee range while the Head is Broken or Destroyed, it must mark an additional HP.  (Źródła: Daktadae: Torso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B834" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C834" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D834" s="8" t="inlineStr">
+        <is>
+          <t>Shake Off</t>
+        </is>
+      </c>
+      <c r="E834" s="8" t="inlineStr">
+        <is>
+          <t>Spend a Fear to throw off foes. All creatures on the colossus must make a Strength Reaction Roll. Targets who fail fall to the ground and must mark a HP. Targets who succeed must mark a Stress.</t>
+        </is>
+      </c>
+      <c r="F834" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G834" s="12" t="n"/>
+      <c r="H834" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I834" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J834" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Torso</t>
+        </is>
+      </c>
+      <c r="K834" t="inlineStr">
+        <is>
+          <t>[Shake Off] Spend a Fear to throw off foes. All creatures on Ikeri must make a Strength Reaction Roll. Targets who fail fall to the ground and must mark a HP. Targets who succeed must mark a Stress.  (Źródła: Ikeri: Torso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B835" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C835" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D835" s="8" t="inlineStr">
+        <is>
+          <t>Kudamat’s Rage</t>
+        </is>
+      </c>
+      <c r="E835" s="8" t="inlineStr">
+        <is>
+          <t>Spend 2 Fear to force all PCs within Very Far range to succeed on a Presence Reaction Roll or become Shaken. While Shaken, they don’t gain Hope on a result with Hope and instead clear the Shaken condition.</t>
+        </is>
+      </c>
+      <c r="F835" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G835" s="12" t="n"/>
+      <c r="H835" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I835" s="12" t="n"/>
+      <c r="J835" s="8" t="inlineStr">
+        <is>
+          <t>Colossus of the Drylands (przykład)</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B836" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C836" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D836" s="8" t="inlineStr">
+        <is>
+          <t>Swatting Pests</t>
+        </is>
+      </c>
+      <c r="E836" s="8" t="inlineStr">
+        <is>
+          <t>When the colossus is attacked by a flying target within Far range, you can make a standard attack against the attacker. On a success, add a d20 to the damage roll and the target is knocked to the ground within Far range.</t>
+        </is>
+      </c>
+      <c r="F836" s="12" t="n"/>
+      <c r="G836" s="12" t="n"/>
+      <c r="H836" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I836" s="12" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="J836" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Framework, Kelir: Framework</t>
+        </is>
+      </c>
+      <c r="K836" t="inlineStr">
+        <is>
+          <t>[Swatting Pests] When Ikeri is attacked by a flying target within Far range, you can make a Peck (Head) or Punch (Arm) standard attack against the attacker. On a success, add a d20 to the damage roll and the target is knocked to the ground at the feet of the colossus.  (Źródła: Ikeri: Framework)</t>
+        </is>
+      </c>
+      <c r="L836" t="inlineStr">
+        <is>
+          <t>[Swatting Pests] When Kelir is attacked by a flying target within Far range, you can make a Pincer (Claws) standard attack against the attacker. On a success, add a d20 to the damage roll and the target is knocked to the ground within Far range.  (Źródła: Kelir: Framework)</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B837" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C837" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D837" s="8" t="inlineStr">
+        <is>
+          <t>Collapsed</t>
+        </is>
+      </c>
+      <c r="E837" s="8" t="inlineStr">
+        <is>
+          <t>When the colossus marks at least 1 HP on all Leg segments, it Collapses. While the colossus is Collapsed, segments that aren’t accessible from the ground can be climbed.</t>
+        </is>
+      </c>
+      <c r="F837" s="12" t="n"/>
+      <c r="G837" s="12" t="n"/>
+      <c r="H837" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I837" s="12" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="J837" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Foreleg ×2, Daktadae: Hindleg ×2, Kelir: Leg ×4</t>
+        </is>
+      </c>
+      <c r="K837" t="inlineStr">
+        <is>
+          <t>[Collapse] If one Foreleg is Destroyed, place a token on this segment. Until it is cleared, Daktadae is Collapsed, allowing PCs to climb directly onto the Torso and Head. If both Forelegs are Destroyed, Daktadae is Collapsed permanently.  (Źródła: Daktadae: Foreleg ×2)</t>
+        </is>
+      </c>
+      <c r="L837" t="inlineStr">
+        <is>
+          <t>[Collapse] If one Hindleg is Destroyed, place a token on this segment. Until it is cleared, Daktadae is Collapsed, allowing PCs to climb directly onto the Torso and Head. If both Hindlegs are Destroyed, Daktadae is Collapsed permanently.  (Źródła: Daktadae: Hindleg ×2)</t>
+        </is>
+      </c>
+      <c r="M837" t="inlineStr">
+        <is>
+          <t>[Full Collapse] Once three Legs are Destroyed, Kelir Collapses and PCs can climb on the Shell and Head from the ground.  (Źródła: Kelir: Leg ×4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B838" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C838" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D838" s="8" t="inlineStr">
+        <is>
+          <t>Colossal Power</t>
+        </is>
+      </c>
+      <c r="E838" s="8" t="inlineStr">
+        <is>
+          <t>When the colossus fails an attack, you gain a Fear.</t>
+        </is>
+      </c>
+      <c r="F838" s="12" t="n"/>
+      <c r="G838" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H838" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I838" s="12" t="inlineStr">
+        <is>
+          <t>1,2,3,4</t>
+        </is>
+      </c>
+      <c r="J838" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Framework, Daktadae: Framework, Poy: Framework, Kelir: Framework</t>
+        </is>
+      </c>
+      <c r="K838" t="inlineStr">
+        <is>
+          <t>[Colossal Power] When Ikeri fails an attack, you gain a Fear.  (Źródła: Ikeri: Framework)</t>
+        </is>
+      </c>
+      <c r="L838" t="inlineStr">
+        <is>
+          <t>[Colossal Power] When Daktadae fails an attack, you gain a Fear.  (Źródła: Daktadae: Framework)</t>
+        </is>
+      </c>
+      <c r="M838" t="inlineStr">
+        <is>
+          <t>[Colossal Power] When Poy fails an attack, you gain a Fear.  (Źródła: Poy: Framework)</t>
+        </is>
+      </c>
+      <c r="N838" t="inlineStr">
+        <is>
+          <t>[Colossal Power] When Kelir fails an attack, you gain a Fear.  (Źródła: Kelir: Framework)</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B839" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C839" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D839" s="8" t="inlineStr">
+        <is>
+          <t>Follow-Up</t>
+        </is>
+      </c>
+      <c r="E839" s="8" t="inlineStr">
+        <is>
+          <t>When the Head succeeds on an attack against a target, it can immediately make an attack against another target it hasn’t attacked during this GM turn.</t>
+        </is>
+      </c>
+      <c r="F839" s="12" t="n"/>
+      <c r="G839" s="12" t="n"/>
+      <c r="H839" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I839" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J839" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B840" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C840" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D840" s="8" t="inlineStr">
+        <is>
+          <t>Massive Stomp</t>
+        </is>
+      </c>
+      <c r="E840" s="8" t="inlineStr">
+        <is>
+          <t>Spend a Fear to make a standard attack with advantage against a group.</t>
+        </is>
+      </c>
+      <c r="F840" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G840" s="12" t="n"/>
+      <c r="H840" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I840" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J840" s="8" t="inlineStr">
+        <is>
+          <t>Ikeri: Leg ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B841" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C841" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D841" s="8" t="inlineStr">
+        <is>
+          <t>Steam-Powered</t>
+        </is>
+      </c>
+      <c r="E841" s="8" t="inlineStr">
+        <is>
+          <t>Scalding fountains of steam erupt from Daktadae’s form. Spotlight any segment to make an attack with a +1 attack modifier against a target on that segment. On a success, deal 2d6+3 physical damage.</t>
+        </is>
+      </c>
+      <c r="F841" s="12" t="n"/>
+      <c r="G841" s="12" t="n"/>
+      <c r="H841" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I841" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J841" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B842" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C842" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D842" s="8" t="inlineStr">
+        <is>
+          <t>Roll</t>
+        </is>
+      </c>
+      <c r="E842" s="8" t="inlineStr">
+        <is>
+          <t>Spend a Fear to have Daktadae drop to the ground and roll. All PCs on Daktadae or within Close range must succeed on an Instinct Reaction Roll (14) or take 2d20+5 physical damage; succeed or fail, the PCs are thrown off Daktadae onto the ground within Melee range of the colossus.</t>
+        </is>
+      </c>
+      <c r="F842" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G842" s="12" t="n"/>
+      <c r="H842" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I842" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J842" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B843" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C843" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D843" s="8" t="inlineStr">
+        <is>
+          <t>Slow Recovery</t>
+        </is>
+      </c>
+      <c r="E843" s="8" t="inlineStr">
+        <is>
+          <t>Clear a token from one Broken or Collapsed segment.</t>
+        </is>
+      </c>
+      <c r="F843" s="12" t="n"/>
+      <c r="G843" s="12" t="n"/>
+      <c r="H843" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I843" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J843" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B844" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C844" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D844" s="8" t="inlineStr">
+        <is>
+          <t>Invulnerable</t>
+        </is>
+      </c>
+      <c r="E844" s="8" t="inlineStr">
+        <is>
+          <t>The Head can only take damage while it’s Broken.</t>
+        </is>
+      </c>
+      <c r="F844" s="12" t="n"/>
+      <c r="G844" s="12" t="n"/>
+      <c r="H844" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I844" s="12" t="inlineStr">
+        <is>
+          <t>2,3</t>
+        </is>
+      </c>
+      <c r="J844" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Head, Poy: Body</t>
+        </is>
+      </c>
+      <c r="K844" t="inlineStr">
+        <is>
+          <t>[Invulnerable] This segment is immune to all damage.  (Źródła: Poy: Body)</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B845" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C845" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D845" s="8" t="inlineStr">
+        <is>
+          <t>Godcleaver</t>
+        </is>
+      </c>
+      <c r="E845" s="8" t="inlineStr">
+        <is>
+          <t>Make a standard attack against a target. On a success, mark a Stress to deal 3d20+12 physical damage instead.</t>
+        </is>
+      </c>
+      <c r="F845" s="12" t="n"/>
+      <c r="G845" s="12" t="n"/>
+      <c r="H845" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I845" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J845" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B846" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C846" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D846" s="8" t="inlineStr">
+        <is>
+          <t>Head Toss</t>
+        </is>
+      </c>
+      <c r="E846" s="8" t="inlineStr">
+        <is>
+          <t>Mark a Stress and make a standard attack against all targets within range who are not on this segment or the Torso. On a success, place 2 tokens on this segment. It is Broken until all tokens are cleared.</t>
+        </is>
+      </c>
+      <c r="F846" s="12" t="n"/>
+      <c r="G846" s="12" t="n"/>
+      <c r="H846" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I846" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J846" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B847" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C847" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D847" s="8" t="inlineStr">
+        <is>
+          <t>Cleaver Recovery</t>
+        </is>
+      </c>
+      <c r="E847" s="8" t="inlineStr">
+        <is>
+          <t>After making a standard attack, place a token on this segment. It is Broken until all tokens are cleared.</t>
+        </is>
+      </c>
+      <c r="F847" s="12" t="n"/>
+      <c r="G847" s="12" t="n"/>
+      <c r="H847" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I847" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J847" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B848" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C848" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D848" s="8" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="E848" s="8" t="inlineStr">
+        <is>
+          <t>The Torso is covered with external rib plates of unbreakable minerals. This segment can’t be damaged unless the Head is currently Broken or Destroyed.</t>
+        </is>
+      </c>
+      <c r="F848" s="12" t="n"/>
+      <c r="G848" s="12" t="n"/>
+      <c r="H848" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I848" s="12" t="inlineStr">
+        <is>
+          <t>2,3</t>
+        </is>
+      </c>
+      <c r="J848" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Torso, Poy: Neck</t>
+        </is>
+      </c>
+      <c r="K848" t="inlineStr">
+        <is>
+          <t>[Protected] Poy’s Neck is protected by swirling magic. The Neck only marks HP from the “Cascade” feature.  (Źródła: Poy: Neck)</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B849" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C849" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D849" s="8" t="inlineStr">
+        <is>
+          <t>Massive Hoof</t>
+        </is>
+      </c>
+      <c r="E849" s="8" t="inlineStr">
+        <is>
+          <t>This segment’s standard attack is made with advantage and can target a group.</t>
+        </is>
+      </c>
+      <c r="F849" s="12" t="n"/>
+      <c r="G849" s="12" t="n"/>
+      <c r="H849" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I849" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J849" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Foreleg ×2, Daktadae: Hindleg ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B850" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C850" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D850" s="8" t="inlineStr">
+        <is>
+          <t>Shake The Earth</t>
+        </is>
+      </c>
+      <c r="E850" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae rears up on their hind legs and slams down, creating a shockwave that knocks back all PCs within Very Close range that aren’t on Daktadae back to Close range and Rattles them until their next roll with Hope. While Rattled, the PC has disadvantage on reaction rolls.</t>
+        </is>
+      </c>
+      <c r="F850" s="12" t="n"/>
+      <c r="G850" s="12" t="n"/>
+      <c r="H850" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I850" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J850" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Foreleg ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B851" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C851" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D851" s="8" t="inlineStr">
+        <is>
+          <t>Backward Kick</t>
+        </is>
+      </c>
+      <c r="E851" s="8" t="inlineStr">
+        <is>
+          <t>All targets within Very Close range behind Daktadae must succeed on an Agility Reaction Roll or take 2d8+10 physical damage.</t>
+        </is>
+      </c>
+      <c r="F851" s="12" t="n"/>
+      <c r="G851" s="12" t="n"/>
+      <c r="H851" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I851" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J851" s="8" t="inlineStr">
+        <is>
+          <t>Daktadae: Hindleg ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B852" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C852" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D852" s="8" t="inlineStr">
+        <is>
+          <t>Strong Winds</t>
+        </is>
+      </c>
+      <c r="E852" s="8" t="inlineStr">
+        <is>
+          <t>While Poy is flying, no other flying creature can come within Close range of Poy without being blown backward by their powerful wings.</t>
+        </is>
+      </c>
+      <c r="F852" s="12" t="n"/>
+      <c r="G852" s="12" t="n"/>
+      <c r="H852" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I852" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J852" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B853" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C853" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D853" s="8" t="inlineStr">
+        <is>
+          <t>Fall Off</t>
+        </is>
+      </c>
+      <c r="E853" s="8" t="inlineStr">
+        <is>
+          <t>When a PC falls off Poy while the colossus is flying, they take 3d20+6 physical damage if they hit the ground.</t>
+        </is>
+      </c>
+      <c r="F853" s="12" t="n"/>
+      <c r="G853" s="12" t="n"/>
+      <c r="H853" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I853" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J853" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B854" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C854" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D854" s="8" t="inlineStr">
+        <is>
+          <t>Bill Trap</t>
+        </is>
+      </c>
+      <c r="E854" s="8" t="inlineStr">
+        <is>
+          <t>Spend a Fear to make an attack against a target on Poy. On a success, the target takes 3d6+6 physical damage and is Trapped inside Poy’s bill until the Head takes Major or greater damage. Poy’s damage thresholds are doubled against damage dealt by Trapped targets.</t>
+        </is>
+      </c>
+      <c r="F854" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G854" s="12" t="n"/>
+      <c r="H854" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I854" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J854" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B855" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C855" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D855" s="8" t="inlineStr">
+        <is>
+          <t>Cascade</t>
+        </is>
+      </c>
+      <c r="E855" s="8" t="inlineStr">
+        <is>
+          <t>When this segment is Destroyed, the Neck must mark 3 HP.</t>
+        </is>
+      </c>
+      <c r="F855" s="12" t="n"/>
+      <c r="G855" s="12" t="n"/>
+      <c r="H855" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I855" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J855" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Head, Poy: Talon ×2, Poy: Tail</t>
+        </is>
+      </c>
+      <c r="K855" t="inlineStr">
+        <is>
+          <t>[Cascade] When this segment is Destroyed, the Neck must mark a HP.  (Źródła: Poy: Talon ×2)</t>
+        </is>
+      </c>
+      <c r="L855" t="inlineStr">
+        <is>
+          <t>[Cascade] When this segment is Destroyed, the Neck must mark 2 HP.  (Źródła: Poy: Tail)</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B856" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C856" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D856" s="8" t="inlineStr">
+        <is>
+          <t>Dust Storm</t>
+        </is>
+      </c>
+      <c r="E856" s="8" t="inlineStr">
+        <is>
+          <t>Poy bats their wings, filling the air and making it much harder to see. Any attacks made by PCs beyond Melee range have disadvantage until the next GM turn.</t>
+        </is>
+      </c>
+      <c r="F856" s="12" t="n"/>
+      <c r="G856" s="12" t="n"/>
+      <c r="H856" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I856" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J856" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Wing ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B857" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C857" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D857" s="8" t="inlineStr">
+        <is>
+          <t>Flap</t>
+        </is>
+      </c>
+      <c r="E857" s="8" t="inlineStr">
+        <is>
+          <t>Poy violently flaps a Wing. Mark a Stress to make an attack against all targets on the Wing. Targets Poy succeeds against take 3d8+4 physical damage and are knocked back onto the Tail. If the Tail is Destroyed, they instead fall off Poy.</t>
+        </is>
+      </c>
+      <c r="F857" s="12" t="n"/>
+      <c r="G857" s="12" t="n"/>
+      <c r="H857" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I857" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J857" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Wing ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B858" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C858" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D858" s="8" t="inlineStr">
+        <is>
+          <t>Dive-Bomb</t>
+        </is>
+      </c>
+      <c r="E858" s="8" t="inlineStr">
+        <is>
+          <t>When this segment is successfully attacked, Poy dive-bombs the attacker and all targets within Very Close range of them. The targets must make an Instinct Reaction Roll. Targets who fail take 2d6+9 physical damage. Targets who succeed can mark a Stress to climb onto one of Poy’s Talons.</t>
+        </is>
+      </c>
+      <c r="F858" s="12" t="n"/>
+      <c r="G858" s="12" t="n"/>
+      <c r="H858" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I858" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J858" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Body</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B859" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C859" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D859" s="8" t="inlineStr">
+        <is>
+          <t>Pick Up</t>
+        </is>
+      </c>
+      <c r="E859" s="8" t="inlineStr">
+        <is>
+          <t>Spend a Fear to make an attack against a target within Melee range. If there’s an additional target within Very Close range of them, you can spotlight both Talons at once and make an attack against both targets instead. On a success, Poy picks up their targets, flies straight upwards, and drops them. If a target hits the ground, they take 5d20+4 physical damage.</t>
+        </is>
+      </c>
+      <c r="F859" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G859" s="12" t="n"/>
+      <c r="H859" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I859" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J859" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Talon ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B860" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C860" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D860" s="8" t="inlineStr">
+        <is>
+          <t>Sweep</t>
+        </is>
+      </c>
+      <c r="E860" s="8" t="inlineStr">
+        <is>
+          <t>Poy’s tail curls up and sweeps across another segment. Spend a Fear to choose another segment and make an attack against all targets on that segment. Targets Poy succeeds against take 3d8+5 physical damage and are knocked back to an adjacent segment of your choice.</t>
+        </is>
+      </c>
+      <c r="F860" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G860" s="12" t="n"/>
+      <c r="H860" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I860" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J860" s="8" t="inlineStr">
+        <is>
+          <t>Poy: Tail</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B861" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C861" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D861" s="8" t="inlineStr">
+        <is>
+          <t>Brood Attack</t>
+        </is>
+      </c>
+      <c r="E861" s="8" t="inlineStr">
+        <is>
+          <t>Spotlight any segment to make an attack with a +6 attack modifier against a PC on that segment as Kelir’s hundred, hundred children swarm the target with their pincers. On a success, deal 4d8 physical damage.</t>
+        </is>
+      </c>
+      <c r="F861" s="12" t="n"/>
+      <c r="G861" s="12" t="n"/>
+      <c r="H861" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I861" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J861" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B862" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C862" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D862" s="8" t="inlineStr">
+        <is>
+          <t>Hateful Gaze</t>
+        </is>
+      </c>
+      <c r="E862" s="8" t="inlineStr">
+        <is>
+          <t>All targets within Far range that Kelir can see must succeed on a Presence Reaction Roll or mark 1d6 Stress as Kelir’s hate tries to consume their mind.</t>
+        </is>
+      </c>
+      <c r="F862" s="12" t="n"/>
+      <c r="G862" s="12" t="n"/>
+      <c r="H862" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I862" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J862" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B863" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C863" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D863" s="8" t="inlineStr">
+        <is>
+          <t>Contagious Fury</t>
+        </is>
+      </c>
+      <c r="E863" s="8" t="inlineStr">
+        <is>
+          <t>All PCs in front of the Head within Far range replace their Hope Die with a d8 the next time they make an action roll as they struggle to keep Kelir’s hatred from consuming them.</t>
+        </is>
+      </c>
+      <c r="F863" s="12" t="n"/>
+      <c r="G863" s="12" t="n"/>
+      <c r="H863" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I863" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J863" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Shell</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B864" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C864" s="12" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D864" s="8" t="inlineStr">
+        <is>
+          <t>Hateful Heart</t>
+        </is>
+      </c>
+      <c r="E864" s="8" t="inlineStr">
+        <is>
+          <t>Kelir’s heart is suspended within the body cavity, connected by thick veins and arteries. The Body Cavity is immune to damage unless her heart is the target of a successful attack. The heart can only be attacked from Far or greater range, or a PC must succeed on an Agility Roll while inside the Body Cavity to reach the heart to make an attack against it within Melee range.</t>
+        </is>
+      </c>
+      <c r="F864" s="12" t="n"/>
+      <c r="G864" s="12" t="n"/>
+      <c r="H864" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I864" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J864" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Body Cavity</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B865" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C865" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D865" s="8" t="inlineStr">
+        <is>
+          <t>Grab and Rend</t>
+        </is>
+      </c>
+      <c r="E865" s="8" t="inlineStr">
+        <is>
+          <t>Make an attack using Kelir’s “Brood Attack” action against a target in the Body Cavity. On a success, spend a Fear to deal double damage and Restrain the target until they’re freed with a successful Strength Roll.</t>
+        </is>
+      </c>
+      <c r="F865" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="G865" s="12" t="n"/>
+      <c r="H865" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I865" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J865" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Body Cavity</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B866" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C866" s="12" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="D866" s="8" t="inlineStr">
+        <is>
+          <t>Protective Swarm</t>
+        </is>
+      </c>
+      <c r="E866" s="8" t="inlineStr">
+        <is>
+          <t>Kelir’s Body Cavity is filled with her children, who protect her heart. A PC who makes an action roll in the Body Cavity must mark a Stress as they fight off Kelir’s children and their shearing pincers.</t>
+        </is>
+      </c>
+      <c r="F866" s="12" t="n"/>
+      <c r="G866" s="12" t="n"/>
+      <c r="H866" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I866" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J866" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Body Cavity</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B867" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C867" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D867" s="8" t="inlineStr">
+        <is>
+          <t>Sever Hope</t>
+        </is>
+      </c>
+      <c r="E867" s="8" t="inlineStr">
+        <is>
+          <t>Make a standard attack against a PC. On a success, mark a Stress to cause the target to lose 1d4 Hope. Gain as many Fear as the Hope lost.</t>
+        </is>
+      </c>
+      <c r="F867" s="12" t="n"/>
+      <c r="G867" s="12" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H867" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I867" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J867" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Claw ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B868" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C868" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D868" s="8" t="inlineStr">
+        <is>
+          <t>Grab &amp; Hurl</t>
+        </is>
+      </c>
+      <c r="E868" s="8" t="inlineStr">
+        <is>
+          <t>Make a standard attack against a target. On a success, instead of dealing damage, hurl the target within Far range in any direction. They must succeed on an Agility Reaction Roll or suffer 3d20 physical damage from the fall.</t>
+        </is>
+      </c>
+      <c r="F868" s="12" t="n"/>
+      <c r="G868" s="12" t="n"/>
+      <c r="H868" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I868" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J868" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Claw ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="13" t="inlineStr">
+        <is>
+          <t>Adversary</t>
+        </is>
+      </c>
+      <c r="B869" s="8" t="inlineStr">
+        <is>
+          <t>Kolosy</t>
+        </is>
+      </c>
+      <c r="C869" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D869" s="8" t="inlineStr">
+        <is>
+          <t>Destructive Scuttle</t>
+        </is>
+      </c>
+      <c r="E869" s="8" t="inlineStr">
+        <is>
+          <t>Mark a Stress to move up to Far range in any direction. All creatures in that path must make an Agility Reaction Roll. Targets who fail take 4d10+6 physical damage and must mark a Stress. Targets who succeed mark a Stress. Kelir can’t use this action if she is Collapsed.</t>
+        </is>
+      </c>
+      <c r="F869" s="12" t="n"/>
+      <c r="G869" s="12" t="n"/>
+      <c r="H869" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I869" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J869" s="8" t="inlineStr">
+        <is>
+          <t>Kelir: Leg ×4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z826"/>
+  <autoFilter ref="A1:Z869"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>